<commit_message>
feat(ui): Cute Scanner Studio UI and Audit Dashboard with presets, health gauge, and instant fixes
</commit_message>
<xml_diff>
--- a/Agile_Template_v0_1.xlsx
+++ b/Agile_Template_v0_1.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -886,6 +886,44 @@
         </is>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>US-12</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>As a developer, I want a complete Scan History &amp; Audit Dashboard to inspect full historical source code, review previous findings, and reload scans.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>US-01, US-06</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Fullstack Dev</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -902,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1550,6 +1588,120 @@
         </is>
       </c>
       <c r="H17" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>US-12</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>T-12.1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Build GET /api/v1/submit/scan/{scan_id} and DELETE /{scan_id} cascading endpoints</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Backend Dev</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>US-12</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>T-12.2</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Implement interactive History Audit Dashboard with code inspector, metrics, and search</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>9</v>
+      </c>
+      <c r="F19" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Frontend Dev</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>US-04</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>T-04.2</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Refactor Java complexity nesting counter to ignore try-with-resources blocks</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Backend Dev</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1566,7 +1718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1720,6 +1872,50 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>Enforced strict JSON schema output formatting and automated code block extraction regex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Try-with-resources constructs in Java were falsely flagged as excessive nesting depth of 5 levels.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Enhanced AST visitor in java_analyzer.py to skip try-with-resources declaration headers in nesting counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Day 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>History view displayed only truncated 2-line code snippets without opening findings or allowing full inspection.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Implemented interactive History Dashboard with detail API integration, multi-tab code viewer, and search filters.</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1919,6 +2115,51 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DevSecOps Team</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Comprehensive AST rule unit testing to detect edge-case false positives early.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Truncating user code snippets in audit logs without full inspection capabilities.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Continuous UI/UX polishing for developer ergonomics and seamless audit flows.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Implemented History Audit Dashboard and refined Java AST SAST rule engine.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>